<commit_message>
actualiza REGLAS_PIE_Y_BONO_PIE.xlsx incorporando reglas actuales implementadas
</commit_message>
<xml_diff>
--- a/REGLAS_PIE_Y_BONO_PIE.xlsx
+++ b/REGLAS_PIE_Y_BONO_PIE.xlsx
@@ -7,16 +7,17 @@
   </bookViews>
   <sheets>
     <sheet name="REGLAS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="REGLAS_ACTUALES_COTIZADOR" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,15 +41,71 @@
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF0000FF"/>
+      <sz val="10"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+      <color indexed="81"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+      <b val="1"/>
+      <color indexed="81"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -77,11 +134,70 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD0E4F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E79"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE699"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAD3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD0E4F7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6DCE4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
@@ -95,8 +211,13 @@
         <fgColor rgb="00D0E4F7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -121,23 +242,51 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00999999"/>
+        <color rgb="FF999999"/>
       </left>
       <right style="thin">
-        <color rgb="00999999"/>
+        <color rgb="FF999999"/>
       </right>
       <top style="thin">
-        <color rgb="00999999"/>
+        <color rgb="FF999999"/>
       </top>
       <bottom style="thin">
-        <color rgb="00999999"/>
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00AAAAAA"/>
+      </left>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -160,16 +309,82 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="8" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="8" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="8" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="7" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="18" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="19" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="20" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="21" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -248,6 +463,34 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Felipe Donoso</author>
+  </authors>
+  <commentList>
+    <comment ref="L2" authorId="0" shapeId="0">
+      <text>
+        <t>Felipe Donoso:
+MAESTRA: Tasación = ValorVenta×(1-%Pie)/(1-%Pie-%BonoPie), BonoPie = Tasación × %BonoPie</t>
+      </text>
+    </comment>
+    <comment ref="L3" authorId="0" shapeId="0">
+      <text>
+        <t>Felipe Donoso:
+INGEVEC: BonoPie = Precio Lista DEPTO × %BonoPie</t>
+      </text>
+    </comment>
+    <comment ref="L4" authorId="0" shapeId="0">
+      <text>
+        <t>Felipe Donoso:
+URMENETA: BonoPie = Precio Lista TOTAL × %BonoPie</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -539,12 +782,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="52" customWidth="1" min="2" max="4"/>
     <col width="65" customWidth="1" min="5" max="5"/>
+    <col width="17" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="16.6640625" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="18.5546875" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="5.5546875" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="11.109375" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="7.6640625" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="13.33203125" bestFit="1" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="22.05" customHeight="1">
@@ -571,6 +821,41 @@
       <c r="E1" s="8" t="inlineStr">
         <is>
           <t>EJEMPLO DE CALCULO (con valores reales)</t>
+        </is>
+      </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>VALOR DEPTO (UF)</t>
+        </is>
+      </c>
+      <c r="G1" s="12" t="inlineStr">
+        <is>
+          <t>VALOR ESTAC (UF)</t>
+        </is>
+      </c>
+      <c r="H1" s="13" t="inlineStr">
+        <is>
+          <t>VALOR BODEGA (UF)</t>
+        </is>
+      </c>
+      <c r="I1" s="13" t="inlineStr">
+        <is>
+          <t>% PIE</t>
+        </is>
+      </c>
+      <c r="J1" s="13" t="inlineStr">
+        <is>
+          <t>% BONO PIE</t>
+        </is>
+      </c>
+      <c r="K1" s="13" t="inlineStr">
+        <is>
+          <t>PIE (UF)</t>
+        </is>
+      </c>
+      <c r="L1" s="13" t="inlineStr">
+        <is>
+          <t>BONO PIE (UF)</t>
         </is>
       </c>
     </row>
@@ -626,6 +911,29 @@
   % Aporte real  = 11.1% de tasacion</t>
         </is>
       </c>
+      <c r="F2" s="14" t="n">
+        <v>3321</v>
+      </c>
+      <c r="G2" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="15" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J2" s="15" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K2" s="16">
+        <f>F2*I2+(G2+H2)*0.2</f>
+        <v/>
+      </c>
+      <c r="L2" s="16">
+        <f>(F2+G2+H2)*(1-I2)/(1-I2-J2)*J2</f>
+        <v/>
+      </c>
     </row>
     <row r="3" ht="180" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -677,6 +985,29 @@
   Credito Hip.   = 4,848.00 - 119.00 - 850.60 = 3,878.40 UF  ($154,546,483)
   Aporte Inmob.  = 850.60 UF  (20% condiciones comerciales)</t>
         </is>
+      </c>
+      <c r="F3" s="17" t="n">
+        <v>4253</v>
+      </c>
+      <c r="G3" s="17" t="n">
+        <v>390</v>
+      </c>
+      <c r="H3" s="17" t="n">
+        <v>205</v>
+      </c>
+      <c r="I3" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="K3" s="19">
+        <f>F3*I3+(G3+H3)*0.2</f>
+        <v/>
+      </c>
+      <c r="L3" s="19">
+        <f>F3*J3</f>
+        <v/>
       </c>
     </row>
     <row r="4" ht="180" customHeight="1">
@@ -729,8 +1060,672 @@
   Aporte Inmob.  = 727.20 UF  (15% condiciones comerciales)</t>
         </is>
       </c>
+      <c r="F4" s="20" t="n">
+        <v>4253</v>
+      </c>
+      <c r="G4" s="20" t="n">
+        <v>390</v>
+      </c>
+      <c r="H4" s="20" t="n">
+        <v>205</v>
+      </c>
+      <c r="I4" s="21" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J4" s="21" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K4" s="22">
+        <f>F4*I4+(G4+H4)*0.2</f>
+        <v/>
+      </c>
+      <c r="L4" s="22">
+        <f>(F4+G4+H4)*J4</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="23" t="inlineStr">
+        <is>
+          <t>REGLAS ACTUALES DE CÁLCULO — COTIZADOR MERCADO PRIMARIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="24" t="inlineStr">
+        <is>
+          <t>REGLA COMÚN — APLICA A TODAS LAS INMOBILIARIAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="25" t="inlineStr">
+        <is>
+          <t>CONCEPTO</t>
+        </is>
+      </c>
+      <c r="B3" s="25" t="inlineStr">
+        <is>
+          <t>FÓRMULA / REGLA</t>
+        </is>
+      </c>
+      <c r="C3" s="25" t="inlineStr">
+        <is>
+          <t>DETALLE</t>
+        </is>
+      </c>
+      <c r="D3" s="25" t="inlineStr">
+        <is>
+          <t>CONDICIÓN</t>
+        </is>
+      </c>
+      <c r="E3" s="25" t="inlineStr">
+        <is>
+          <t>FUENTE EN CÓDIGO</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>PIE TOTAL</t>
+        </is>
+      </c>
+      <c r="B4" s="27" t="inlineStr">
+        <is>
+          <t>Pie Depto + Pie Conjuntos</t>
+        </is>
+      </c>
+      <c r="C4" s="27" t="inlineStr">
+        <is>
+          <t>Pie Depto = Precio Desc. Depto x %Pie
+Pie Conjuntos = Precio Lista (Estac+Bodega) x 20%</t>
+        </is>
+      </c>
+      <c r="D4" s="27" t="inlineStr">
+        <is>
+          <t>Bienes conjuntos SIEMPRE 20%,
+independiente del %Pie del depto</t>
+        </is>
+      </c>
+      <c r="E4" s="27" t="inlineStr">
+        <is>
+          <t>cotizador.ts: pieTotalDeptoUF
++ pieTotalConjuntosUF</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="26" t="inlineStr">
+        <is>
+          <t>% PIE DEFAULT EN UI</t>
+        </is>
+      </c>
+      <c r="B5" s="27" t="inlineStr">
+        <is>
+          <t>max(0, 20% - %BonoPie)</t>
+        </is>
+      </c>
+      <c r="C5" s="27" t="inlineStr">
+        <is>
+          <t>Ejemplo: BonoPie=20% -&gt; Pie=0%
+         BonoPie=15% -&gt; Pie=5%
+         BonoPie=0%  -&gt; Pie=10%</t>
+        </is>
+      </c>
+      <c r="D5" s="27" t="inlineStr">
+        <is>
+          <t>Solo cuando existe bono pie
+en condiciones comerciales</t>
+        </is>
+      </c>
+      <c r="E5" s="27" t="inlineStr">
+        <is>
+          <t>PanelCotizacion.tsx: useState
+(unidad.bonoPie &gt; 0 ? ...)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>UPFRONT PROMESA</t>
+        </is>
+      </c>
+      <c r="B6" s="27" t="inlineStr">
+        <is>
+          <t>Bloqueado en 0%
+cuando hay bono pie</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>Si bonoPie &gt; 0 en condiciones
+comerciales: control deshabilitado
+y valor = 0%</t>
+        </is>
+      </c>
+      <c r="D6" s="27" t="inlineStr">
+        <is>
+          <t>Aplica a todas las inmobiliarias
+que tienen bono pie</t>
+        </is>
+      </c>
+      <c r="E6" s="27" t="inlineStr">
+        <is>
+          <t>PanelCotizacion.tsx:
+disabled={unidad.bonoPie &gt; 0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>DETECCIÓN DE INMOBILIARIA</t>
+        </is>
+      </c>
+      <c r="B7" s="27" t="inlineStr">
+        <is>
+          <t>Por nombre de alianza
+(case-insensitive)</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>getTipoCalculoBono(alianza):
+  "maestra"  -&gt; regla Maestra
+  "urmeneta" -&gt; regla Urmeneta
+  resto      -&gt; regla INGEVEC/default</t>
+        </is>
+      </c>
+      <c r="D7" s="27" t="inlineStr">
+        <is>
+          <t>Comparacion con .includes()
+sobre el nombre de alianza</t>
+        </is>
+      </c>
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>cotizadorConfig.ts:
+getTipoCalculoBono()
+getLtvMaxPct()</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>REGLAS ESPECÍFICAS POR INMOBILIARIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="28" t="inlineStr">
+        <is>
+          <t>Los campos en VERDE son comunes; los diferenciadores están resaltados por color de inmobiliaria</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="25" t="inlineStr">
+        <is>
+          <t>CONCEPTO</t>
+        </is>
+      </c>
+      <c r="B11" s="25" t="inlineStr">
+        <is>
+          <t>MAESTRA</t>
+        </is>
+      </c>
+      <c r="C11" s="25" t="inlineStr">
+        <is>
+          <t>INGEVEC (y resto default)</t>
+        </is>
+      </c>
+      <c r="D11" s="25" t="inlineStr">
+        <is>
+          <t>URMENETA</t>
+        </is>
+      </c>
+      <c r="E11" s="25" t="inlineStr">
+        <is>
+          <t>NOTAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="65" customHeight="1">
+      <c r="A12" s="29" t="inlineStr">
+        <is>
+          <t>Detección</t>
+        </is>
+      </c>
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>alianza.includes("maestra")</t>
+        </is>
+      </c>
+      <c r="C12" s="31" t="inlineStr">
+        <is>
+          <t>cualquier alias no reconocido
+como Maestra ni Urmeneta</t>
+        </is>
+      </c>
+      <c r="D12" s="32" t="inlineStr">
+        <is>
+          <t>alianza.includes("urmeneta")</t>
+        </is>
+      </c>
+      <c r="E12" s="33" t="inlineStr">
+        <is>
+          <t>getTipoCalculoBono()
+en cotizadorConfig.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="65" customHeight="1">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>tipoCalculoBono</t>
+        </is>
+      </c>
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t>'maestra'</t>
+        </is>
+      </c>
+      <c r="C13" s="31" t="inlineStr">
+        <is>
+          <t>'precio-lista-depto'</t>
+        </is>
+      </c>
+      <c r="D13" s="32" t="inlineStr">
+        <is>
+          <t>'precio-lista-total'</t>
+        </is>
+      </c>
+      <c r="E13" s="33" t="inlineStr">
+        <is>
+          <t>Valor pasado al motor
+como input.tipoCalculoBono</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="65" customHeight="1">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>LTV máximo banco
+(ltvMaxPct)</t>
+        </is>
+      </c>
+      <c r="B14" s="30" t="inlineStr">
+        <is>
+          <t>0.80  (80%)</t>
+        </is>
+      </c>
+      <c r="C14" s="27" t="inlineStr">
+        <is>
+          <t>1.0  (sin límite especial)</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="inlineStr">
+        <is>
+          <t>1.0  (sin límite especial)</t>
+        </is>
+      </c>
+      <c r="E14" s="33" t="inlineStr">
+        <is>
+          <t>getLtvMaxPct(alianza)
+en cotizadorConfig.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="65" customHeight="1">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>Base de cálculo
+Bono Pie</t>
+        </is>
+      </c>
+      <c r="B15" s="30" t="inlineStr">
+        <is>
+          <t>TASACIÓN BANCO
+(% se aplica sobre tasación,
+no sobre valor venta)</t>
+        </is>
+      </c>
+      <c r="C15" s="31" t="inlineStr">
+        <is>
+          <t>PRECIO LISTA DEPTO
+(solo departamento,
+excluye bienes conjuntos)</t>
+        </is>
+      </c>
+      <c r="D15" s="32" t="inlineStr">
+        <is>
+          <t>PRECIO LISTA TOTAL
+(depto + estac + bodega)</t>
+        </is>
+      </c>
+      <c r="E15" s="33" t="inlineStr">
+        <is>
+          <t>Diferencia clave
+entre inmobiliarias</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="65" customHeight="1">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>Fórmula Bono Pie (UF)</t>
+        </is>
+      </c>
+      <c r="B16" s="30" t="inlineStr">
+        <is>
+          <t>D36: Tasación × %BonoPie
+(Tasación se despeja primero en D35)</t>
+        </is>
+      </c>
+      <c r="C16" s="31" t="inlineStr">
+        <is>
+          <t>PrecioListaDepto × %BonoPie</t>
+        </is>
+      </c>
+      <c r="D16" s="32" t="inlineStr">
+        <is>
+          <t>PrecioListaTotal × %BonoPie</t>
+        </is>
+      </c>
+      <c r="E16" s="33" t="inlineStr"/>
+    </row>
+    <row r="17" ht="65" customHeight="1">
+      <c r="A17" s="29" t="inlineStr">
+        <is>
+          <t>Fórmula Tasación Banco</t>
+        </is>
+      </c>
+      <c r="B17" s="30" t="inlineStr">
+        <is>
+          <t>D35: ValorVenta × (1-pie)
+     / (1 - pie - bono%)
+[Excel Calculadora BP+Mutuo]</t>
+        </is>
+      </c>
+      <c r="C17" s="27" t="inlineStr">
+        <is>
+          <t>ValorVenta + BonoPieUF</t>
+        </is>
+      </c>
+      <c r="D17" s="27" t="inlineStr">
+        <is>
+          <t>ValorVenta + BonoPieUF</t>
+        </is>
+      </c>
+      <c r="E17" s="33" t="inlineStr">
+        <is>
+          <t>Maestra: fórmula
+inversa (tasación despejada)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="65" customHeight="1">
+      <c r="A18" s="29" t="inlineStr">
+        <is>
+          <t>Fórmula
+Crédito Hipotecario</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="inlineStr">
+        <is>
+          <t>Tasación × 80%
+(LTV máximo especial)</t>
+        </is>
+      </c>
+      <c r="C18" s="27" t="inlineStr">
+        <is>
+          <t>ValorVenta - PieTotal - AporteInmob</t>
+        </is>
+      </c>
+      <c r="D18" s="27" t="inlineStr">
+        <is>
+          <t>ValorVenta - PieTotal - AporteInmob</t>
+        </is>
+      </c>
+      <c r="E18" s="33" t="inlineStr">
+        <is>
+          <t>Maestra tiene regla
+exclusiva de LTV 80%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="65" customHeight="1">
+      <c r="A19" s="29" t="inlineStr">
+        <is>
+          <t>Aporte Inmobiliaria (UF)</t>
+        </is>
+      </c>
+      <c r="B19" s="30" t="inlineStr">
+        <is>
+          <t>Tasación - PieTotal - CréditoHip
+(residual, absorbe diferencia LTV)</t>
+        </is>
+      </c>
+      <c r="C19" s="27" t="inlineStr">
+        <is>
+          <t>BonoPieUF calculado</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
+        <is>
+          <t>BonoPieUF calculado</t>
+        </is>
+      </c>
+      <c r="E19" s="33" t="inlineStr"/>
+    </row>
+    <row r="20" ht="65" customHeight="1">
+      <c r="A20" s="29" t="inlineStr">
+        <is>
+          <t>% display Aporte
+(en tabla cotización)</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>Calculado real:
+saldoAporte / Tasación
+(puede diferir del % nominal)</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="inlineStr">
+        <is>
+          <t>%BonoPie de condiciones
+comerciales (nominal)</t>
+        </is>
+      </c>
+      <c r="D20" s="32" t="inlineStr">
+        <is>
+          <t>%BonoPie de condiciones
+comerciales (nominal)</t>
+        </is>
+      </c>
+      <c r="E20" s="33" t="inlineStr">
+        <is>
+          <t>Solo Maestra muestra
+% real calculado</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="24" t="inlineStr">
+        <is>
+          <t>COMO AGREGAR UNA NUEVA INMOBILIARIA CON REGLA ESPECIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="25" t="inlineStr">
+        <is>
+          <t>PASO</t>
+        </is>
+      </c>
+      <c r="B23" s="25" t="inlineStr">
+        <is>
+          <t>ACCIÓN</t>
+        </is>
+      </c>
+      <c r="C23" s="25" t="inlineStr">
+        <is>
+          <t>DETALLE</t>
+        </is>
+      </c>
+      <c r="D23" s="25" t="inlineStr">
+        <is>
+          <t>CONDICIÓN</t>
+        </is>
+      </c>
+      <c r="E23" s="25" t="inlineStr">
+        <is>
+          <t>ARCHIVO / LINEA</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="60" customHeight="1">
+      <c r="A24" s="29" t="inlineStr">
+        <is>
+          <t>Paso 1 — Definir tipo
+de cálculo</t>
+        </is>
+      </c>
+      <c r="B24" s="27" t="inlineStr">
+        <is>
+          <t>Editar getTipoCalculoBono()
+en lib/config/cotizadorConfig.ts</t>
+        </is>
+      </c>
+      <c r="C24" s="33" t="inlineStr">
+        <is>
+          <t>Agregar:
+  if (norm.includes('nombre_alianza'))
+    return 'precio-lista-depto' | 'precio-lista-total' | 'maestra'</t>
+        </is>
+      </c>
+      <c r="D24" s="33" t="inlineStr"/>
+      <c r="E24" s="33" t="inlineStr">
+        <is>
+          <t>cotizadorConfig.ts
+lineas 85-90</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="60" customHeight="1">
+      <c r="A25" s="29" t="inlineStr">
+        <is>
+          <t>Paso 2 — Definir LTV
+(si aplica)</t>
+        </is>
+      </c>
+      <c r="B25" s="27" t="inlineStr">
+        <is>
+          <t>Editar getLtvMaxPct()
+en lib/config/cotizadorConfig.ts</t>
+        </is>
+      </c>
+      <c r="C25" s="33" t="inlineStr">
+        <is>
+          <t>Si el banco aplica LTV especial:
+  return alianza.includes('x') ? LTV_X : 1.0</t>
+        </is>
+      </c>
+      <c r="D25" s="33" t="inlineStr">
+        <is>
+          <t>Solo si el LTV difiere del estándar</t>
+        </is>
+      </c>
+      <c r="E25" s="33" t="inlineStr">
+        <is>
+          <t>cotizadorConfig.ts
+lineas 72-74</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="60" customHeight="1">
+      <c r="A26" s="29" t="inlineStr">
+        <is>
+          <t>Paso 3 — Lógica de
+cálculo nueva (si aplica)</t>
+        </is>
+      </c>
+      <c r="B26" s="27" t="inlineStr">
+        <is>
+          <t>Agregar bloque en
+lib/calculators/cotizador.ts</t>
+        </is>
+      </c>
+      <c r="C26" s="33" t="inlineStr">
+        <is>
+          <t>En el bloque if/else de
+tipoCalculoBono:
+  } else if (tipoCalculoBono === 'nueva') {</t>
+        </is>
+      </c>
+      <c r="D26" s="33" t="inlineStr">
+        <is>
+          <t>Solo si la fórmula difiere
+de las 3 existentes</t>
+        </is>
+      </c>
+      <c r="E26" s="33" t="inlineStr">
+        <is>
+          <t>cotizador.ts
+lineas 220-250</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="60" customHeight="1">
+      <c r="A27" s="29" t="inlineStr">
+        <is>
+          <t>Paso 4 — Documentar</t>
+        </is>
+      </c>
+      <c r="B27" s="27" t="inlineStr">
+        <is>
+          <t>Actualizar REGLAS_PIE_Y_BONO_PIE.xlsx
+y MAESTRO_DESARROLLO_COTIZADOR.md</t>
+        </is>
+      </c>
+      <c r="C27" s="33" t="inlineStr"/>
+      <c r="D27" s="33" t="inlineStr"/>
+      <c r="E27" s="33" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A9:E9"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
corrige cálculo Maestra y desbloquea Upfront para todas las inmobiliarias
- Maestra: aporte inmobiliaria usa pieTotalDeptoUF (no conjuntos) → 414,69 UF correcto
- Agrega pieCreditoHipUF al resultado para mostrar pie correcto por tipo inmobiliaria
- Desbloquea Upfront Promesa (%) para todas las inmobiliarias, default 2%
- Actualiza REGLAS_PIE_Y_BONO_PIE.xlsx con hoja REGLAS_ACTUALES_COTIZADOR

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/REGLAS_PIE_Y_BONO_PIE.xlsx
+++ b/REGLAS_PIE_Y_BONO_PIE.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AI\cotizador-web-mp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{456361D2-E97B-447D-9849-96DA4C6CE8B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{077B6ABA-3C22-40DF-A8E2-235AC8E789C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="REGLAS" sheetId="1" r:id="rId1"/>
     <sheet name="REGLAS_ACTUALES_COTIZADOR" sheetId="2" r:id="rId2"/>
     <sheet name="REGLAS_ACTUALES_COTIZADOR_POR_I" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -471,7 +472,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="126">
   <si>
     <t>INMOBILIARIA</t>
   </si>
@@ -1407,6 +1408,82 @@
     <xf numFmtId="0" fontId="15" fillId="21" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="17" fillId="11" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="17" fillId="11" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="17" fillId="11" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="17" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="17" fillId="11" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="17" fillId="12" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="17" fillId="12" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="17" fillId="12" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="17" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="17" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="17" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="17" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="17" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1416,82 +1493,6 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="17" fillId="11" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="17" fillId="11" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="17" fillId="11" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="17" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="17" fillId="11" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="17" fillId="12" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="17" fillId="12" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="17" fillId="12" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="17" fillId="12" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="17" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="17" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="17" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="17" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1510,10 +1511,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1852,25 +1849,25 @@
       <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="33" t="s">
+      <c r="F1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="33" t="s">
+      <c r="G1" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="34" t="s">
+      <c r="H1" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="34" t="s">
+      <c r="I1" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="34" t="s">
+      <c r="J1" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="34" t="s">
+      <c r="K1" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="34" t="s">
+      <c r="L1" s="30" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2010,22 +2007,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="58" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
     </row>
     <row r="2" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="55" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
+      <c r="B2" s="56"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
     </row>
     <row r="3" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="21" t="s">
@@ -2113,22 +2110,22 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="29" t="s">
+      <c r="A9" s="55" t="s">
         <v>51</v>
       </c>
-      <c r="B9" s="30"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="30"/>
-      <c r="E9" s="30"/>
+      <c r="B9" s="56"/>
+      <c r="C9" s="56"/>
+      <c r="D9" s="56"/>
+      <c r="E9" s="56"/>
     </row>
     <row r="10" spans="1:5" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="31" t="s">
+      <c r="A10" s="57" t="s">
         <v>52</v>
       </c>
-      <c r="B10" s="30"/>
-      <c r="C10" s="30"/>
-      <c r="D10" s="30"/>
-      <c r="E10" s="30"/>
+      <c r="B10" s="56"/>
+      <c r="C10" s="56"/>
+      <c r="D10" s="56"/>
+      <c r="E10" s="56"/>
     </row>
     <row r="11" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="21" t="s">
@@ -2297,13 +2294,13 @@
       </c>
     </row>
     <row r="22" spans="1:5" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="29" t="s">
+      <c r="A22" s="55" t="s">
         <v>93</v>
       </c>
-      <c r="B22" s="30"/>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="30"/>
+      <c r="B22" s="56"/>
+      <c r="C22" s="56"/>
+      <c r="D22" s="56"/>
+      <c r="E22" s="56"/>
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="21" t="s">
@@ -2413,204 +2410,204 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35" t="s">
+      <c r="B1" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="35" t="s">
+      <c r="C1" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="35" t="s">
+      <c r="D1" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="36" t="s">
+      <c r="E1" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="37" t="s">
+      <c r="F1" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="37" t="s">
+      <c r="G1" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="38" t="s">
+      <c r="H1" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="38" t="s">
+      <c r="I1" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="38" t="s">
+      <c r="J1" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="38" t="s">
+      <c r="K1" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="39" t="s">
+      <c r="L1" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="39" t="s">
+      <c r="M1" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="N1" s="39" t="s">
+      <c r="N1" s="35" t="s">
         <v>114</v>
       </c>
-      <c r="O1" s="38" t="s">
+      <c r="O1" s="34" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="41" t="s">
+      <c r="B2" s="37" t="s">
         <v>116</v>
       </c>
-      <c r="C2" s="41" t="s">
+      <c r="C2" s="37" t="s">
         <v>117</v>
       </c>
-      <c r="D2" s="41" t="s">
+      <c r="D2" s="37" t="s">
         <v>118</v>
       </c>
-      <c r="E2" s="41" t="s">
+      <c r="E2" s="37" t="s">
         <v>119</v>
       </c>
-      <c r="F2" s="42">
+      <c r="F2" s="38">
         <v>5000</v>
       </c>
-      <c r="G2" s="42">
+      <c r="G2" s="38">
         <v>200</v>
       </c>
-      <c r="H2" s="42">
+      <c r="H2" s="38">
         <v>100</v>
       </c>
-      <c r="I2" s="43">
+      <c r="I2" s="39">
         <v>0.1</v>
       </c>
-      <c r="J2" s="43">
+      <c r="J2" s="39">
         <v>0.1</v>
       </c>
-      <c r="K2" s="44">
+      <c r="K2" s="40">
         <f>F2*I2 + (G2+H2)*0.2</f>
         <v>560</v>
       </c>
-      <c r="L2" s="45">
+      <c r="L2" s="41">
         <f>M2*J2</f>
         <v>596.25</v>
       </c>
-      <c r="M2" s="46">
+      <c r="M2" s="42">
         <f>(F2+G2+H2)*(1-I2) / (1-I2-J2)</f>
         <v>5962.5</v>
       </c>
-      <c r="N2" s="44">
+      <c r="N2" s="40">
         <f>M2*0.8</f>
         <v>4770</v>
       </c>
-      <c r="O2" s="45">
+      <c r="O2" s="41">
         <f>M2-K2-N2</f>
         <v>632.5</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="47" t="s">
+      <c r="A3" s="43" t="s">
         <v>120</v>
       </c>
-      <c r="B3" s="48" t="s">
+      <c r="B3" s="44" t="s">
         <v>116</v>
       </c>
-      <c r="C3" s="48" t="s">
+      <c r="C3" s="44" t="s">
         <v>121</v>
       </c>
-      <c r="D3" s="48" t="s">
+      <c r="D3" s="44" t="s">
         <v>122</v>
       </c>
-      <c r="E3" s="48" t="s">
+      <c r="E3" s="44" t="s">
         <v>123</v>
       </c>
-      <c r="F3" s="49">
+      <c r="F3" s="45">
         <v>5000</v>
       </c>
-      <c r="G3" s="49">
+      <c r="G3" s="45">
         <v>200</v>
       </c>
-      <c r="H3" s="49">
+      <c r="H3" s="45">
         <v>100</v>
       </c>
-      <c r="I3" s="50">
+      <c r="I3" s="46">
         <v>0.1</v>
       </c>
-      <c r="J3" s="50">
+      <c r="J3" s="46">
         <v>0.1</v>
       </c>
-      <c r="K3" s="51">
+      <c r="K3" s="47">
         <f>F3*I3 + (G3+H3)*0.2</f>
         <v>560</v>
       </c>
-      <c r="L3" s="51">
+      <c r="L3" s="47">
         <f>F3*J3</f>
         <v>500</v>
       </c>
-      <c r="M3" s="51">
+      <c r="M3" s="47">
         <f>(F3+G3+H3)+L3</f>
         <v>5800</v>
       </c>
-      <c r="N3" s="51">
+      <c r="N3" s="47">
         <f>(F3+G3+H3)-K3-L3</f>
         <v>4240</v>
       </c>
-      <c r="O3" s="52">
+      <c r="O3" s="48">
         <f>L3</f>
         <v>500</v>
       </c>
     </row>
     <row r="4" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="53" t="s">
+      <c r="A4" s="49" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="54" t="s">
+      <c r="B4" s="50" t="s">
         <v>116</v>
       </c>
-      <c r="C4" s="54" t="s">
+      <c r="C4" s="50" t="s">
         <v>124</v>
       </c>
-      <c r="D4" s="54" t="s">
+      <c r="D4" s="50" t="s">
         <v>122</v>
       </c>
-      <c r="E4" s="54" t="s">
+      <c r="E4" s="50" t="s">
         <v>125</v>
       </c>
-      <c r="F4" s="55">
+      <c r="F4" s="51">
         <v>5000</v>
       </c>
-      <c r="G4" s="55">
+      <c r="G4" s="51">
         <v>200</v>
       </c>
-      <c r="H4" s="55">
+      <c r="H4" s="51">
         <v>100</v>
       </c>
-      <c r="I4" s="56">
+      <c r="I4" s="52">
         <v>0.1</v>
       </c>
-      <c r="J4" s="56">
+      <c r="J4" s="52">
         <v>0.1</v>
       </c>
-      <c r="K4" s="57">
+      <c r="K4" s="53">
         <f>F4*I4 + (G4+H4)*0.2</f>
         <v>560</v>
       </c>
-      <c r="L4" s="57">
+      <c r="L4" s="53">
         <f>(F4+G4+H4)*J4</f>
         <v>530</v>
       </c>
-      <c r="M4" s="57">
+      <c r="M4" s="53">
         <f>(F4+G4+H4)+L4</f>
         <v>5830</v>
       </c>
-      <c r="N4" s="57">
+      <c r="N4" s="53">
         <f>(F4+G4+H4)-K4-L4</f>
         <v>4210</v>
       </c>
-      <c r="O4" s="58">
+      <c r="O4" s="54">
         <f>L4</f>
         <v>530</v>
       </c>
@@ -2619,4 +2616,22 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B36E29F-7595-4353-9580-7BD031296451}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>